<commit_message>
feat : add new tables to dataset
</commit_message>
<xml_diff>
--- a/data/applications.xlsx
+++ b/data/applications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yassi\job-search-analytics\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE2ED81D-475C-4D82-913B-6FE205B09F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B27AEBD1-CE4F-476B-B895-9918471505CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{CAA645E2-DF17-4657-914C-F65452DF32D8}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
   <si>
     <t>ID</t>
   </si>
@@ -81,13 +81,25 @@
     <t>24/04/2026</t>
   </si>
   <si>
-    <t>Linkedin</t>
-  </si>
-  <si>
     <t>Envoyé</t>
   </si>
   <si>
     <t>Non</t>
+  </si>
+  <si>
+    <t>LinkedIn</t>
+  </si>
+  <si>
+    <t>Secteur</t>
+  </si>
+  <si>
+    <t>Temps_Réponse</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>Industrie</t>
   </si>
 </sst>
 </file>
@@ -117,7 +129,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -140,144 +152,17 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -592,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919FD5C4-7F7C-4C2A-B1FC-7A3004547902}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
@@ -602,42 +487,49 @@
     <col min="6" max="7" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="6">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -653,19 +545,23 @@
         <v>17</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="7"/>
+        <v>19</v>
+      </c>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="6">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -681,44 +577,52 @@
         <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="7"/>
-    </row>
-    <row r="4" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="8">
-        <v>3</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="1"/>
+      <c r="I4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="10"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
feat : update job applications dataset with new entries
</commit_message>
<xml_diff>
--- a/data/applications.xlsx
+++ b/data/applications.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yassi\job-search-analytics\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B27AEBD1-CE4F-476B-B895-9918471505CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F09F5C5-C384-44CE-82DA-ED679B9BCB97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{CAA645E2-DF17-4657-914C-F65452DF32D8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Applications" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Applications!$A$1:$K$5</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="26">
   <si>
     <t>ID</t>
   </si>
@@ -78,34 +81,40 @@
     <t>Paris</t>
   </si>
   <si>
-    <t>24/04/2026</t>
-  </si>
-  <si>
     <t>Envoyé</t>
   </si>
   <si>
-    <t>Non</t>
-  </si>
-  <si>
     <t>LinkedIn</t>
   </si>
   <si>
     <t>Secteur</t>
   </si>
   <si>
-    <t>Temps_Réponse</t>
-  </si>
-  <si>
     <t>IT</t>
   </si>
   <si>
     <t>Industrie</t>
+  </si>
+  <si>
+    <t>GRDF</t>
+  </si>
+  <si>
+    <t>Entretien</t>
+  </si>
+  <si>
+    <t>Energie</t>
+  </si>
+  <si>
+    <t>Saint-Denis</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -162,7 +171,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -477,20 +486,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919FD5C4-7F7C-4C2A-B1FC-7A3004547902}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -521,46 +530,44 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>21</v>
+      <c r="K1" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>17</v>
+        <v>25</v>
+      </c>
+      <c r="E2" s="3">
+        <v>46106</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
+      </c>
+      <c r="H2" s="3">
+        <v>46113</v>
+      </c>
+      <c r="I2" s="1">
+        <v>1</v>
       </c>
       <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1" t="s">
-        <v>23</v>
+      <c r="K2" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -573,26 +580,25 @@
       <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="3">
+        <v>46136</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>18</v>
-      </c>
       <c r="H3" s="1"/>
-      <c r="I3" s="1" t="s">
-        <v>19</v>
+      <c r="I3" s="1">
+        <v>0</v>
       </c>
       <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1" t="s">
-        <v>24</v>
+      <c r="K3" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -605,26 +611,59 @@
       <c r="D4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="3">
+        <v>46136</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="H4" s="1"/>
+      <c r="I4" s="1">
+        <v>0</v>
+      </c>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="1" t="s">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3">
+        <v>46136</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1" t="s">
-        <v>23</v>
+      <c r="G5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K5">
+    <sortCondition ref="A1:A5"/>
+  </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat : status update of an application
</commit_message>
<xml_diff>
--- a/data/applications.xlsx
+++ b/data/applications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yassi\job-search-analytics\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F09F5C5-C384-44CE-82DA-ED679B9BCB97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E2E7770-99E7-44C8-9AC5-8A3EF1E65FF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{CAA645E2-DF17-4657-914C-F65452DF32D8}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
   <si>
     <t>ID</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>Saint-Denis</t>
+  </si>
+  <si>
+    <t>Refus</t>
   </si>
 </sst>
 </file>
@@ -113,9 +116,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -129,6 +132,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -138,7 +149,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -161,22 +172,350 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="14">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -187,6 +526,26 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}" name="Table1" displayName="Table1" ref="A1:K5" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11" totalsRowBorderDxfId="10">
+  <autoFilter ref="A1:K5" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{F9F6E859-0E4E-4AB1-AB82-AE8C68095E3C}" name="ID" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{5AC9CDA5-8818-4959-80C1-F4CA3CDCFE9E}" name="Entreprise" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{820BFA22-51B0-4843-AADB-9E5D1E0CD1AB}" name="Poste" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{04D827DB-3217-4C69-B1C0-00AA2639625A}" name="Lieu" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{37C391F2-9459-4E6F-91CB-FCC9DE5CE7AC}" name="Date_Candidature" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{CF125D61-14E6-4A1C-B426-A9316483785F}" name="Source" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{5E494642-05B8-44F7-BEEC-D3AB0412C070}" name="Statut" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{FE6ED1E8-A124-4415-9932-0481A9E189D7}" name="Date_reponse"/>
+    <tableColumn id="9" xr3:uid="{2E05DE79-3F14-4817-9F22-5BC14AA187B7}" name="Relance" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{A711714D-3A92-4105-B404-C89598D2444C}" name="Notes" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{EC7DC286-2B37-4A16-929D-FA4B107DAA5E}" name="Secteur" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -492,50 +851,52 @@
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.109375" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" customWidth="1"/>
     <col min="7" max="7" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5546875" customWidth="1"/>
+    <col min="9" max="9" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" customWidth="1"/>
+    <col min="11" max="11" width="9.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="12" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -547,7 +908,7 @@
       <c r="D2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="2">
         <v>46106</v>
       </c>
       <c r="F2" s="1" t="s">
@@ -556,19 +917,19 @@
       <c r="G2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="2">
         <v>46113</v>
       </c>
       <c r="I2" s="1">
         <v>1</v>
       </c>
       <c r="J2" s="1"/>
-      <c r="K2" s="1" t="s">
+      <c r="K2" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -580,7 +941,7 @@
       <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <v>46136</v>
       </c>
       <c r="F3" s="1" t="s">
@@ -589,17 +950,17 @@
       <c r="G3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="1"/>
+      <c r="H3" s="2"/>
       <c r="I3" s="1">
         <v>0</v>
       </c>
       <c r="J3" s="1"/>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -611,52 +972,54 @@
       <c r="D4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <v>46136</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>18</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" s="1"/>
+        <v>26</v>
+      </c>
+      <c r="H4" s="2">
+        <v>46139</v>
+      </c>
       <c r="I4" s="1">
         <v>0</v>
       </c>
       <c r="J4" s="1"/>
-      <c r="K4" s="1" t="s">
+      <c r="K4" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+      <c r="A5" s="5">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="7">
         <v>46136</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1">
+      <c r="H5" s="6"/>
+      <c r="I5" s="6">
         <v>0</v>
       </c>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1" t="s">
+      <c r="J5" s="6"/>
+      <c r="K5" s="8" t="s">
         <v>20</v>
       </c>
     </row>
@@ -666,5 +1029,8 @@
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat : New applications added
</commit_message>
<xml_diff>
--- a/data/applications.xlsx
+++ b/data/applications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yassi\job-search-analytics\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E2E7770-99E7-44C8-9AC5-8A3EF1E65FF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8717CC4-B7DF-44F9-AF88-4FF3035375C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{CAA645E2-DF17-4657-914C-F65452DF32D8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Applications" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Applications!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Applications!$A$1:$K$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="35">
   <si>
     <t>ID</t>
   </si>
@@ -109,6 +109,30 @@
   </si>
   <si>
     <t>Refus</t>
+  </si>
+  <si>
+    <t>Sephora</t>
+  </si>
+  <si>
+    <t>Data Analyst</t>
+  </si>
+  <si>
+    <t>Linkedin</t>
+  </si>
+  <si>
+    <t>Retail</t>
+  </si>
+  <si>
+    <t>Thales</t>
+  </si>
+  <si>
+    <t>Bouygues Telecom</t>
+  </si>
+  <si>
+    <t>Meudon</t>
+  </si>
+  <si>
+    <t>Telecom</t>
   </si>
 </sst>
 </file>
@@ -272,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -288,6 +312,7 @@
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -529,8 +554,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}" name="Table1" displayName="Table1" ref="A1:K5" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11" totalsRowBorderDxfId="10">
-  <autoFilter ref="A1:K5" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}" name="Table1" displayName="Table1" ref="A1:K8" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11" totalsRowBorderDxfId="10">
+  <autoFilter ref="A1:K8" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{F9F6E859-0E4E-4AB1-AB82-AE8C68095E3C}" name="ID" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{5AC9CDA5-8818-4959-80C1-F4CA3CDCFE9E}" name="Entreprise" dataDxfId="8"/>
@@ -845,7 +870,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919FD5C4-7F7C-4C2A-B1FC-7A3004547902}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
@@ -1023,6 +1048,99 @@
         <v>20</v>
       </c>
     </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="7">
+        <v>46140</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="13"/>
+      <c r="I6" s="6">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6"/>
+      <c r="K6" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="7">
+        <v>46140</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="13"/>
+      <c r="I7" s="6">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6"/>
+      <c r="K7" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="7">
+        <v>46140</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="13"/>
+      <c r="I8" s="6">
+        <v>0</v>
+      </c>
+      <c r="J8" s="6"/>
+      <c r="K8" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K5">
     <sortCondition ref="A1:A5"/>

</xml_diff>

<commit_message>
feat: new database entries and Dashboard modifications
</commit_message>
<xml_diff>
--- a/data/applications.xlsx
+++ b/data/applications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yassi\job-search-analytics\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8717CC4-B7DF-44F9-AF88-4FF3035375C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{683463E3-E16F-4CAC-8118-3B612EEEA0CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{CAA645E2-DF17-4657-914C-F65452DF32D8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Applications" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Applications!$A$1:$K$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Applications!$A$1:$K$9</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
   <si>
     <t>ID</t>
   </si>
@@ -133,6 +133,9 @@
   </si>
   <si>
     <t>Telecom</t>
+  </si>
+  <si>
+    <t>Green Yellow</t>
   </si>
 </sst>
 </file>
@@ -312,7 +315,7 @@
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -554,8 +557,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}" name="Table1" displayName="Table1" ref="A1:K8" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11" totalsRowBorderDxfId="10">
-  <autoFilter ref="A1:K8" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}" name="Table1" displayName="Table1" ref="A1:K9" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11" totalsRowBorderDxfId="10">
+  <autoFilter ref="A1:K9" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{F9F6E859-0E4E-4AB1-AB82-AE8C68095E3C}" name="ID" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{5AC9CDA5-8818-4959-80C1-F4CA3CDCFE9E}" name="Entreprise" dataDxfId="8"/>
@@ -870,7 +873,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919FD5C4-7F7C-4C2A-B1FC-7A3004547902}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
@@ -1070,7 +1073,6 @@
       <c r="G6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="13"/>
       <c r="I6" s="6">
         <v>0</v>
       </c>
@@ -1101,7 +1103,6 @@
       <c r="G7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="13"/>
       <c r="I7" s="6">
         <v>0</v>
       </c>
@@ -1132,13 +1133,45 @@
       <c r="G8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="13"/>
       <c r="I8" s="6">
         <v>0</v>
       </c>
       <c r="J8" s="6"/>
       <c r="K8" s="8" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="7">
+        <v>46140</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9" s="13">
+        <v>46142</v>
+      </c>
+      <c r="I9" s="6">
+        <v>0</v>
+      </c>
+      <c r="J9" s="6"/>
+      <c r="K9" s="8" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: updating database and dashboard
</commit_message>
<xml_diff>
--- a/data/applications.xlsx
+++ b/data/applications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yassi\job-search-analytics\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{683463E3-E16F-4CAC-8118-3B612EEEA0CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5944807-7713-4401-9FC3-DA1B6E62A7BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{CAA645E2-DF17-4657-914C-F65452DF32D8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Applications" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Applications!$A$1:$K$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Applications!$A$1:$K$19</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="51">
   <si>
     <t>ID</t>
   </si>
@@ -126,9 +126,6 @@
     <t>Thales</t>
   </si>
   <si>
-    <t>Bouygues Telecom</t>
-  </si>
-  <si>
     <t>Meudon</t>
   </si>
   <si>
@@ -136,6 +133,54 @@
   </si>
   <si>
     <t>Green Yellow</t>
+  </si>
+  <si>
+    <t>MBDA</t>
+  </si>
+  <si>
+    <t>Le Plessis-Robinson</t>
+  </si>
+  <si>
+    <t>Gennevilliers</t>
+  </si>
+  <si>
+    <t>Guyancourt</t>
+  </si>
+  <si>
+    <t>RTE</t>
+  </si>
+  <si>
+    <t>La Défense</t>
+  </si>
+  <si>
+    <t>Construction</t>
+  </si>
+  <si>
+    <t>Capgemini</t>
+  </si>
+  <si>
+    <t>Issy-les-Moulineaux</t>
+  </si>
+  <si>
+    <t>Dior</t>
+  </si>
+  <si>
+    <t>Renault</t>
+  </si>
+  <si>
+    <t>Luxe</t>
+  </si>
+  <si>
+    <t>Automobile</t>
+  </si>
+  <si>
+    <t>Chanel</t>
+  </si>
+  <si>
+    <t>Louis Vuitton</t>
+  </si>
+  <si>
+    <t>Bouygues</t>
   </si>
 </sst>
 </file>
@@ -299,7 +344,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -315,12 +360,13 @@
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="15">
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -372,6 +418,9 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -483,6 +532,7 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right style="thin">
@@ -507,15 +557,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -523,6 +564,15 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -557,17 +607,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}" name="Table1" displayName="Table1" ref="A1:K9" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11" totalsRowBorderDxfId="10">
-  <autoFilter ref="A1:K9" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}" name="Table1" displayName="Table1" ref="A1:K19" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="12" tableBorderDxfId="13" totalsRowBorderDxfId="11">
+  <autoFilter ref="A1:K19" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{F9F6E859-0E4E-4AB1-AB82-AE8C68095E3C}" name="ID" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{5AC9CDA5-8818-4959-80C1-F4CA3CDCFE9E}" name="Entreprise" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{820BFA22-51B0-4843-AADB-9E5D1E0CD1AB}" name="Poste" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{04D827DB-3217-4C69-B1C0-00AA2639625A}" name="Lieu" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{37C391F2-9459-4E6F-91CB-FCC9DE5CE7AC}" name="Date_Candidature" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{CF125D61-14E6-4A1C-B426-A9316483785F}" name="Source" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{5E494642-05B8-44F7-BEEC-D3AB0412C070}" name="Statut" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{FE6ED1E8-A124-4415-9932-0481A9E189D7}" name="Date_reponse"/>
+    <tableColumn id="1" xr3:uid="{F9F6E859-0E4E-4AB1-AB82-AE8C68095E3C}" name="ID" dataDxfId="10">
+      <calculatedColumnFormula>ROW()-ROW(Table1[#Headers])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{5AC9CDA5-8818-4959-80C1-F4CA3CDCFE9E}" name="Entreprise" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{820BFA22-51B0-4843-AADB-9E5D1E0CD1AB}" name="Poste" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{04D827DB-3217-4C69-B1C0-00AA2639625A}" name="Lieu" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{37C391F2-9459-4E6F-91CB-FCC9DE5CE7AC}" name="Date_Candidature" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{CF125D61-14E6-4A1C-B426-A9316483785F}" name="Source" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{5E494642-05B8-44F7-BEEC-D3AB0412C070}" name="Statut" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{FE6ED1E8-A124-4415-9932-0481A9E189D7}" name="Date_reponse" dataDxfId="3"/>
     <tableColumn id="9" xr3:uid="{2E05DE79-3F14-4817-9F22-5BC14AA187B7}" name="Relance" dataDxfId="2"/>
     <tableColumn id="10" xr3:uid="{A711714D-3A92-4105-B404-C89598D2444C}" name="Notes" dataDxfId="1"/>
     <tableColumn id="11" xr3:uid="{EC7DC286-2B37-4A16-929D-FA4B107DAA5E}" name="Secteur" dataDxfId="0"/>
@@ -873,10 +925,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919FD5C4-7F7C-4C2A-B1FC-7A3004547902}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.109375" customWidth="1"/>
@@ -885,7 +937,7 @@
     <col min="8" max="8" width="14.5546875" customWidth="1"/>
     <col min="9" max="9" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.77734375" customWidth="1"/>
-    <col min="11" max="11" width="9.21875" customWidth="1"/>
+    <col min="11" max="11" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -925,6 +977,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
+        <f>ROW()-ROW(Table1[#Headers])</f>
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -958,6 +1011,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
+        <f>ROW()-ROW(Table1[#Headers])</f>
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -989,6 +1043,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
+        <f>ROW()-ROW(Table1[#Headers])</f>
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -1022,6 +1077,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
@@ -1042,7 +1098,7 @@
       <c r="G5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="6"/>
+      <c r="H5" s="7"/>
       <c r="I5" s="6">
         <v>0</v>
       </c>
@@ -1053,6 +1109,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
@@ -1073,6 +1130,7 @@
       <c r="G6" s="6" t="s">
         <v>17</v>
       </c>
+      <c r="H6" s="13"/>
       <c r="I6" s="6">
         <v>0</v>
       </c>
@@ -1083,6 +1141,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -1103,6 +1162,7 @@
       <c r="G7" s="6" t="s">
         <v>17</v>
       </c>
+      <c r="H7" s="13"/>
       <c r="I7" s="6">
         <v>0</v>
       </c>
@@ -1113,16 +1173,17 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>28</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E8" s="7">
         <v>46140</v>
@@ -1133,20 +1194,22 @@
       <c r="G8" s="6" t="s">
         <v>17</v>
       </c>
+      <c r="H8" s="13"/>
       <c r="I8" s="6">
         <v>0</v>
       </c>
       <c r="J8" s="6"/>
       <c r="K8" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>13</v>
@@ -1172,6 +1235,326 @@
       <c r="J9" s="6"/>
       <c r="K9" s="8" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="7">
+        <v>46146</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="14"/>
+      <c r="I10" s="6">
+        <v>0</v>
+      </c>
+      <c r="J10" s="6"/>
+      <c r="K10" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="7">
+        <v>46146</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="14"/>
+      <c r="I11" s="6">
+        <v>0</v>
+      </c>
+      <c r="J11" s="6"/>
+      <c r="K11" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="7">
+        <v>46146</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="14"/>
+      <c r="I12" s="6">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6"/>
+      <c r="K12" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>12</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" s="7">
+        <v>46146</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" s="14"/>
+      <c r="I13" s="6">
+        <v>0</v>
+      </c>
+      <c r="J13" s="6"/>
+      <c r="K13" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="7">
+        <v>46146</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="14"/>
+      <c r="I14" s="6">
+        <v>0</v>
+      </c>
+      <c r="J14" s="6"/>
+      <c r="K14" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>14</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15" s="7">
+        <v>46146</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="14"/>
+      <c r="I15" s="6">
+        <v>0</v>
+      </c>
+      <c r="J15" s="6"/>
+      <c r="K15" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>15</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16" s="7">
+        <v>46146</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" s="14"/>
+      <c r="I16" s="6">
+        <v>0</v>
+      </c>
+      <c r="J16" s="6"/>
+      <c r="K16" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>16</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" s="7">
+        <v>46146</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="14"/>
+      <c r="I17" s="6">
+        <v>0</v>
+      </c>
+      <c r="J17" s="6"/>
+      <c r="K17" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>17</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="7">
+        <v>46146</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="14"/>
+      <c r="I18" s="6">
+        <v>0</v>
+      </c>
+      <c r="J18" s="6"/>
+      <c r="K18" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="5">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>18</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="7">
+        <v>46146</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" s="14"/>
+      <c r="I19" s="6">
+        <v>0</v>
+      </c>
+      <c r="J19" s="6"/>
+      <c r="K19" s="8" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1180,8 +1563,9 @@
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add new applications
</commit_message>
<xml_diff>
--- a/data/applications.xlsx
+++ b/data/applications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yassi\job-search-analytics\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5944807-7713-4401-9FC3-DA1B6E62A7BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7304FDD-037A-4973-834D-48B63E6A9DB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{CAA645E2-DF17-4657-914C-F65452DF32D8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Applications" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Applications!$A$1:$K$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Applications!$A$1:$K$29</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="64">
   <si>
     <t>ID</t>
   </si>
@@ -181,6 +181,45 @@
   </si>
   <si>
     <t>Bouygues</t>
+  </si>
+  <si>
+    <t>Safran</t>
+  </si>
+  <si>
+    <t>Accenture</t>
+  </si>
+  <si>
+    <t>Massy</t>
+  </si>
+  <si>
+    <t>Aéronautique</t>
+  </si>
+  <si>
+    <t>#REF</t>
+  </si>
+  <si>
+    <t>Data Scientist Junior</t>
+  </si>
+  <si>
+    <t>Ingénieur Data &amp; développeur BI</t>
+  </si>
+  <si>
+    <t>Ingénieur en science des données CATIA</t>
+  </si>
+  <si>
+    <t>Développement d'algorithmes d'analyse de données de vol</t>
+  </si>
+  <si>
+    <t>Moissy-Cramayel</t>
+  </si>
+  <si>
+    <t>Corbeille-Essone</t>
+  </si>
+  <si>
+    <t>Apprenti-e Data Analyst F/H</t>
+  </si>
+  <si>
+    <t>Data Analyst Supply Chain MRO</t>
   </si>
 </sst>
 </file>
@@ -190,7 +229,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -208,6 +247,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -341,50 +388,81 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
     <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -397,12 +475,11 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -415,15 +492,63 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -436,12 +561,11 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -454,13 +578,11 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -473,26 +595,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -557,6 +659,15 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -564,15 +675,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -607,22 +709,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}" name="Table1" displayName="Table1" ref="A1:K19" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="12" tableBorderDxfId="13" totalsRowBorderDxfId="11">
-  <autoFilter ref="A1:K19" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{F9F6E859-0E4E-4AB1-AB82-AE8C68095E3C}" name="ID" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}" name="Table1" displayName="Table1" ref="A1:L29" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13" totalsRowBorderDxfId="12">
+  <autoFilter ref="A1:L29" xr:uid="{A0B28C6D-6477-43D9-B373-D8255AFA4F9E}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{F9F6E859-0E4E-4AB1-AB82-AE8C68095E3C}" name="ID" dataDxfId="11">
       <calculatedColumnFormula>ROW()-ROW(Table1[#Headers])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{5AC9CDA5-8818-4959-80C1-F4CA3CDCFE9E}" name="Entreprise" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{5AC9CDA5-8818-4959-80C1-F4CA3CDCFE9E}" name="Entreprise" dataDxfId="10"/>
     <tableColumn id="3" xr3:uid="{820BFA22-51B0-4843-AADB-9E5D1E0CD1AB}" name="Poste" dataDxfId="8"/>
     <tableColumn id="4" xr3:uid="{04D827DB-3217-4C69-B1C0-00AA2639625A}" name="Lieu" dataDxfId="7"/>
     <tableColumn id="5" xr3:uid="{37C391F2-9459-4E6F-91CB-FCC9DE5CE7AC}" name="Date_Candidature" dataDxfId="6"/>
     <tableColumn id="6" xr3:uid="{CF125D61-14E6-4A1C-B426-A9316483785F}" name="Source" dataDxfId="5"/>
     <tableColumn id="7" xr3:uid="{5E494642-05B8-44F7-BEEC-D3AB0412C070}" name="Statut" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{FE6ED1E8-A124-4415-9932-0481A9E189D7}" name="Date_reponse" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{2E05DE79-3F14-4817-9F22-5BC14AA187B7}" name="Relance" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{A711714D-3A92-4105-B404-C89598D2444C}" name="Notes" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{EC7DC286-2B37-4A16-929D-FA4B107DAA5E}" name="Secteur" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{FE6ED1E8-A124-4415-9932-0481A9E189D7}" name="Date_reponse" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{2E05DE79-3F14-4817-9F22-5BC14AA187B7}" name="Relance" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{A711714D-3A92-4105-B404-C89598D2444C}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{EC7DC286-2B37-4A16-929D-FA4B107DAA5E}" name="Secteur" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{FD78B42C-76B8-438B-809F-071A743F09A7}" name="#REF" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -925,636 +1028,1002 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919FD5C4-7F7C-4C2A-B1FC-7A3004547902}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.109375" customWidth="1"/>
-    <col min="6" max="6" width="8.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" customWidth="1"/>
+    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5546875" customWidth="1"/>
+    <col min="8" max="8" width="11.109375" customWidth="1"/>
     <col min="9" max="9" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.77734375" customWidth="1"/>
     <col min="11" max="11" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="49.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="8" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="3">
+      <c r="L1" s="14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="16">
         <v>46106</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="1" t="s">
+      <c r="F2" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="16">
         <v>46113</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="15">
         <v>1</v>
       </c>
-      <c r="J2" s="1"/>
-      <c r="K2" s="4" t="s">
+      <c r="J2" s="15"/>
+      <c r="K2" s="18" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
+      <c r="L2" s="10"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="16">
         <v>46136</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="1">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1"/>
-      <c r="K3" s="4" t="s">
+      <c r="F3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="16"/>
+      <c r="I3" s="15">
+        <v>0</v>
+      </c>
+      <c r="J3" s="15"/>
+      <c r="K3" s="18" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
+      <c r="L3" s="1"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="16">
         <v>46136</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="1" t="s">
+      <c r="F4" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="16">
         <v>46139</v>
       </c>
-      <c r="I4" s="1">
-        <v>0</v>
-      </c>
-      <c r="J4" s="1"/>
-      <c r="K4" s="4" t="s">
+      <c r="I4" s="15">
+        <v>0</v>
+      </c>
+      <c r="J4" s="15"/>
+      <c r="K4" s="18" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="5">
+      <c r="L4" s="1"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="17">
         <v>46136</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" s="7"/>
-      <c r="I5" s="6">
-        <v>0</v>
-      </c>
-      <c r="J5" s="6"/>
-      <c r="K5" s="8" t="s">
+      <c r="F5" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="16"/>
+      <c r="I5" s="19">
+        <v>0</v>
+      </c>
+      <c r="J5" s="19"/>
+      <c r="K5" s="20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="5">
+      <c r="L5" s="12" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="17">
         <v>46140</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H6" s="13"/>
-      <c r="I6" s="6">
-        <v>0</v>
-      </c>
-      <c r="J6" s="6"/>
-      <c r="K6" s="8" t="s">
+      <c r="G6" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="16"/>
+      <c r="I6" s="19">
+        <v>0</v>
+      </c>
+      <c r="J6" s="19"/>
+      <c r="K6" s="20" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="5">
+      <c r="L6" s="1"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="17">
         <v>46140</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="13"/>
-      <c r="I7" s="6">
-        <v>0</v>
-      </c>
-      <c r="J7" s="6"/>
-      <c r="K7" s="8" t="s">
+      <c r="G7" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="16"/>
+      <c r="I7" s="19">
+        <v>0</v>
+      </c>
+      <c r="J7" s="19"/>
+      <c r="K7" s="20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="5">
+      <c r="L7" s="1"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="17">
         <v>46140</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="13"/>
-      <c r="I8" s="6">
-        <v>0</v>
-      </c>
-      <c r="J8" s="6"/>
-      <c r="K8" s="8" t="s">
+      <c r="G8" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="16"/>
+      <c r="I8" s="19">
+        <v>0</v>
+      </c>
+      <c r="J8" s="19"/>
+      <c r="K8" s="20" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="5">
+      <c r="L8" s="1"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="17">
         <v>46140</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="6" t="s">
+      <c r="F9" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="H9" s="13">
+      <c r="H9" s="16">
         <v>46142</v>
       </c>
-      <c r="I9" s="6">
-        <v>0</v>
-      </c>
-      <c r="J9" s="6"/>
-      <c r="K9" s="8" t="s">
+      <c r="I9" s="19">
+        <v>0</v>
+      </c>
+      <c r="J9" s="19"/>
+      <c r="K9" s="20" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="5">
+      <c r="L9" s="1"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="17">
         <v>46146</v>
       </c>
-      <c r="F10" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="14"/>
-      <c r="I10" s="6">
-        <v>0</v>
-      </c>
-      <c r="J10" s="6"/>
-      <c r="K10" s="8" t="s">
+      <c r="F10" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="16">
+        <v>46147</v>
+      </c>
+      <c r="I10" s="19">
+        <v>0</v>
+      </c>
+      <c r="J10" s="19"/>
+      <c r="K10" s="20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="5">
+      <c r="L10" s="1"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="17">
         <v>46146</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" s="14"/>
-      <c r="I11" s="6">
-        <v>0</v>
-      </c>
-      <c r="J11" s="6"/>
-      <c r="K11" s="8" t="s">
+      <c r="F11" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="16"/>
+      <c r="I11" s="19">
+        <v>0</v>
+      </c>
+      <c r="J11" s="19"/>
+      <c r="K11" s="20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="5">
+      <c r="L11" s="1"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>11</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="17">
         <v>46146</v>
       </c>
-      <c r="F12" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12" s="14"/>
-      <c r="I12" s="6">
-        <v>0</v>
-      </c>
-      <c r="J12" s="6"/>
-      <c r="K12" s="8" t="s">
+      <c r="F12" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="16"/>
+      <c r="I12" s="19">
+        <v>0</v>
+      </c>
+      <c r="J12" s="19"/>
+      <c r="K12" s="20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="5">
+      <c r="L12" s="1"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>12</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="17">
         <v>46146</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H13" s="14"/>
-      <c r="I13" s="6">
-        <v>0</v>
-      </c>
-      <c r="J13" s="6"/>
-      <c r="K13" s="8" t="s">
+      <c r="F13" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" s="16"/>
+      <c r="I13" s="19">
+        <v>0</v>
+      </c>
+      <c r="J13" s="19"/>
+      <c r="K13" s="20" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="5">
+      <c r="L13" s="1"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>13</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="7">
+      <c r="E14" s="17">
         <v>46146</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="14"/>
-      <c r="I14" s="6">
-        <v>0</v>
-      </c>
-      <c r="J14" s="6"/>
-      <c r="K14" s="8" t="s">
+      <c r="F14" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="16"/>
+      <c r="I14" s="19">
+        <v>0</v>
+      </c>
+      <c r="J14" s="19"/>
+      <c r="K14" s="20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="5">
+      <c r="L14" s="1"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>14</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="17">
         <v>46146</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H15" s="14"/>
-      <c r="I15" s="6">
-        <v>0</v>
-      </c>
-      <c r="J15" s="6"/>
-      <c r="K15" s="8" t="s">
+      <c r="F15" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="16"/>
+      <c r="I15" s="19">
+        <v>0</v>
+      </c>
+      <c r="J15" s="19"/>
+      <c r="K15" s="20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="5">
+      <c r="L15" s="1"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>15</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E16" s="7">
+      <c r="E16" s="17">
         <v>46146</v>
       </c>
-      <c r="F16" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H16" s="14"/>
-      <c r="I16" s="6">
-        <v>0</v>
-      </c>
-      <c r="J16" s="6"/>
-      <c r="K16" s="8" t="s">
+      <c r="F16" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" s="16"/>
+      <c r="I16" s="19">
+        <v>0</v>
+      </c>
+      <c r="J16" s="19"/>
+      <c r="K16" s="20" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="5">
+      <c r="L16" s="1"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
         <f>ROW()-ROW(Table1[#Headers])</f>
         <v>16</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="7">
+      <c r="E17" s="17">
         <v>46146</v>
       </c>
-      <c r="F17" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H17" s="14"/>
-      <c r="I17" s="6">
-        <v>0</v>
-      </c>
-      <c r="J17" s="6"/>
-      <c r="K17" s="8" t="s">
+      <c r="F17" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G17" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="16"/>
+      <c r="I17" s="19">
+        <v>0</v>
+      </c>
+      <c r="J17" s="19"/>
+      <c r="K17" s="20" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A18" s="5">
-        <f>ROW()-ROW(Table1[#Headers])</f>
-        <v>17</v>
-      </c>
-      <c r="B18" s="6" t="s">
+      <c r="L17" s="1"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>17</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E18" s="7">
+      <c r="E18" s="17">
         <v>46146</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H18" s="14"/>
-      <c r="I18" s="6">
-        <v>0</v>
-      </c>
-      <c r="J18" s="6"/>
-      <c r="K18" s="8" t="s">
+      <c r="F18" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="16"/>
+      <c r="I18" s="19">
+        <v>0</v>
+      </c>
+      <c r="J18" s="19"/>
+      <c r="K18" s="20" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" s="5">
-        <f>ROW()-ROW(Table1[#Headers])</f>
-        <v>18</v>
-      </c>
-      <c r="B19" s="6" t="s">
+      <c r="L18" s="1"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>18</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="17">
         <v>46146</v>
       </c>
-      <c r="F19" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H19" s="14"/>
-      <c r="I19" s="6">
-        <v>0</v>
-      </c>
-      <c r="J19" s="6"/>
-      <c r="K19" s="8" t="s">
+      <c r="F19" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" s="16"/>
+      <c r="I19" s="19">
+        <v>0</v>
+      </c>
+      <c r="J19" s="19"/>
+      <c r="K19" s="20" t="s">
         <v>46</v>
+      </c>
+      <c r="L19" s="1"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20" s="9">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="17">
+        <v>46147</v>
+      </c>
+      <c r="F20" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G20" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H20" s="16"/>
+      <c r="I20" s="19">
+        <v>0</v>
+      </c>
+      <c r="J20" s="19"/>
+      <c r="K20" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="L20" s="1"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A21" s="9">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" s="17">
+        <v>46147</v>
+      </c>
+      <c r="F21" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" s="16"/>
+      <c r="I21" s="19">
+        <v>0</v>
+      </c>
+      <c r="J21" s="19"/>
+      <c r="K21" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="L21" s="1"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A22" s="9">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>21</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22" s="17">
+        <v>46147</v>
+      </c>
+      <c r="F22" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G22" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="16"/>
+      <c r="I22" s="19">
+        <v>0</v>
+      </c>
+      <c r="J22" s="19"/>
+      <c r="K22" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="L22" s="1"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A23" s="9">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>22</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23" s="17">
+        <v>46147</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H23" s="16"/>
+      <c r="I23" s="19">
+        <v>0</v>
+      </c>
+      <c r="J23" s="19"/>
+      <c r="K23" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="L23" s="1"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24" s="9">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>23</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="E24" s="17">
+        <v>46147</v>
+      </c>
+      <c r="F24" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G24" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H24" s="16"/>
+      <c r="I24" s="19">
+        <v>0</v>
+      </c>
+      <c r="J24" s="19"/>
+      <c r="K24" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="L24" s="1"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25" s="9">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>24</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E25" s="17">
+        <v>46147</v>
+      </c>
+      <c r="F25" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G25" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" s="16"/>
+      <c r="I25" s="19">
+        <v>0</v>
+      </c>
+      <c r="J25" s="19"/>
+      <c r="K25" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="L25" s="11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A26" s="9">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>25</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="17">
+        <v>46147</v>
+      </c>
+      <c r="F26" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G26" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H26" s="16"/>
+      <c r="I26" s="19">
+        <v>0</v>
+      </c>
+      <c r="J26" s="19"/>
+      <c r="K26" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="L26" s="13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A27" s="9">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D27" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="17">
+        <v>46147</v>
+      </c>
+      <c r="F27" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G27" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H27" s="16"/>
+      <c r="I27" s="19">
+        <v>0</v>
+      </c>
+      <c r="J27" s="19"/>
+      <c r="K27" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="L27" s="13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A28" s="9">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>27</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="E28" s="17">
+        <v>46147</v>
+      </c>
+      <c r="F28" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G28" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" s="17"/>
+      <c r="I28" s="19">
+        <v>0</v>
+      </c>
+      <c r="J28" s="19"/>
+      <c r="K28" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="L28" s="13" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A29" s="9">
+        <f>ROW()-ROW(Table1[#Headers])</f>
+        <v>28</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D29" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="E29" s="17">
+        <v>46147</v>
+      </c>
+      <c r="F29" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H29" s="17"/>
+      <c r="I29" s="19">
+        <v>0</v>
+      </c>
+      <c r="J29" s="19"/>
+      <c r="K29" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="L29" s="13" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1562,10 +2031,18 @@
     <sortCondition ref="A1:A5"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="L25" r:id="rId1" display="Poste" xr:uid="{F55B037D-DFDB-4933-AA1F-2955D88E257B}"/>
+    <hyperlink ref="L5" r:id="rId2" xr:uid="{6F4433D6-A790-4F49-92F4-3AA5D963591D}"/>
+    <hyperlink ref="L27" r:id="rId3" xr:uid="{E655547D-C443-4928-839C-ADD896D196AA}"/>
+    <hyperlink ref="L26" r:id="rId4" xr:uid="{98DB469C-D4D4-4D24-A43E-313E372FF5EB}"/>
+    <hyperlink ref="L28" r:id="rId5" display=" Data Analyst Supply Chain MRO" xr:uid="{8698C37C-D41E-42D6-A7F2-71328C34E490}"/>
+    <hyperlink ref="L29" r:id="rId6" xr:uid="{EBAC8C9D-7E30-407B-A87D-90AA4FA25628}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
+  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId7"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>